<commit_message>
Adequação do código para submissão, incluindo: * Geração de planilhas em excel, correspondentes tanto às tabelas quanto às figuras. * Geração de gráficos em .svg * Adição de comentários no código, para melhorar a legibilidade
</commit_message>
<xml_diff>
--- a/output/basegrafico4.xlsx
+++ b/output/basegrafico4.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -370,11 +370,6 @@
           <t>contagem</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>livro</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -388,12 +383,6 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral em Geral</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -407,14 +396,6 @@
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Das Condutas Vedadas
-aos Agentes Públicos
-em Campanhas
-Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -428,11 +409,6 @@
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Disposições Finais</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -446,12 +422,6 @@
       <c r="C5">
         <v>8</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Da Fiscalização das
-Eleições</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -465,15 +435,6 @@
       <c r="C6">
         <v>6</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Do Sistema
-Eletrônico de
-Votação e da
-Totalização dos
-Votos</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -487,12 +448,6 @@
       <c r="C7">
         <v>4</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Da Fiscalização das
-Eleições</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -506,15 +461,6 @@
       <c r="C8">
         <v>5</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Do Sistema
-Eletrônico de
-Votação e da
-Totalização dos
-Votos</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -528,14 +474,6 @@
       <c r="C9">
         <v>19</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Da Arrecadação
-e da Aplicação
-de Recursos nas
-Campanhas Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -549,12 +487,6 @@
       <c r="C10">
         <v>5</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Da Prestação de
-Contas</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -568,12 +500,6 @@
       <c r="C11">
         <v>9</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral em Geral</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -587,13 +513,6 @@
       <c r="C12">
         <v>16</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral mediante
-outdoors</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -607,13 +526,6 @@
       <c r="C13">
         <v>2</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral na
-Imprensa</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -627,13 +539,6 @@
       <c r="C14">
         <v>4</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral no Rádio e
-na Televisão</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -647,14 +552,6 @@
       <c r="C15">
         <v>1</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Das Condutas Vedadas
-aos Agentes Públicos
-em Campanhas
-Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -668,13 +565,6 @@
       <c r="C16">
         <v>1</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Das Pesquisas
-e Testes
-Pré-Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -688,11 +578,6 @@
       <c r="C17">
         <v>5</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Disposições Finais</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -706,14 +591,6 @@
       <c r="C18">
         <v>14</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Da Arrecadação
-e da Aplicação
-de Recursos nas
-Campanhas Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -727,12 +604,6 @@
       <c r="C19">
         <v>15</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Da Prestação de
-Contas</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -746,12 +617,6 @@
       <c r="C20">
         <v>37</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral em Geral</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -765,13 +630,6 @@
       <c r="C21">
         <v>3</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral na
-Imprensa</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -785,13 +643,6 @@
       <c r="C22">
         <v>24</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral no Rádio e
-na Televisão</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -805,11 +656,6 @@
       <c r="C23">
         <v>2</v>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Das Coligações</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -823,14 +669,6 @@
       <c r="C24">
         <v>8</v>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Das Condutas Vedadas
-aos Agentes Públicos
-em Campanhas
-Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -844,13 +682,6 @@
       <c r="C25">
         <v>3</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Das Convenções
-para a Escolha de
-Candidatos</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -864,13 +695,6 @@
       <c r="C26">
         <v>1</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Das Pesquisas
-e Testes
-Pré-Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -884,11 +708,6 @@
       <c r="C27">
         <v>17</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Disposições Finais</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -902,12 +721,6 @@
       <c r="C28">
         <v>1</v>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Disposições
-Transitórias</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -921,12 +734,6 @@
       <c r="C29">
         <v>5</v>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Do Direito de
-Resposta</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -940,12 +747,6 @@
       <c r="C30">
         <v>17</v>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Do Registro de
-Candidatos</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -959,12 +760,6 @@
       <c r="C31">
         <v>25</v>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Propaganda na
-Internet</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -978,11 +773,6 @@
       <c r="C32">
         <v>6</v>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Disposições Finais</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -996,14 +786,6 @@
       <c r="C33">
         <v>10</v>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Da Arrecadação
-e da Aplicação
-de Recursos nas
-Campanhas Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -1017,12 +799,6 @@
       <c r="C34">
         <v>1</v>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Da Fiscalização das
-Eleições</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -1036,12 +812,6 @@
       <c r="C35">
         <v>10</v>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Da Prestação de
-Contas</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -1055,12 +825,6 @@
       <c r="C36">
         <v>22</v>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral em Geral</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -1074,13 +838,6 @@
       <c r="C37">
         <v>12</v>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral no Rádio e
-na Televisão</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -1094,11 +851,6 @@
       <c r="C38">
         <v>1</v>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Das Coligações</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -1112,13 +864,6 @@
       <c r="C39">
         <v>1</v>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Das Convenções
-para a Escolha de
-Candidatos</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -1132,13 +877,6 @@
       <c r="C40">
         <v>3</v>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Das Pesquisas
-e Testes
-Pré-Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -1152,11 +890,6 @@
       <c r="C41">
         <v>16</v>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Disposições Finais</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -1170,12 +903,6 @@
       <c r="C42">
         <v>1</v>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Do Direito de
-Resposta</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -1189,12 +916,6 @@
       <c r="C43">
         <v>4</v>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Do Registro de
-Candidatos</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -1208,12 +929,6 @@
       <c r="C44">
         <v>3</v>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Propaganda na
-Internet</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -1227,15 +942,6 @@
       <c r="C45">
         <v>3</v>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Do Sistema
-Eletrônico de
-Votação e da
-Totalização dos
-Votos</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -1249,14 +955,6 @@
       <c r="C46">
         <v>41</v>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Da Arrecadação
-e da Aplicação
-de Recursos nas
-Campanhas Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -1270,12 +968,6 @@
       <c r="C47">
         <v>22</v>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Da Prestação de
-Contas</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -1289,12 +981,6 @@
       <c r="C48">
         <v>12</v>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral em Geral</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -1308,13 +994,6 @@
       <c r="C49">
         <v>44</v>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral no Rádio e
-na Televisão</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -1328,14 +1007,6 @@
       <c r="C50">
         <v>1</v>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Das Condutas Vedadas
-aos Agentes Públicos
-em Campanhas
-Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -1349,13 +1020,6 @@
       <c r="C51">
         <v>2</v>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Das Convenções
-para a Escolha de
-Candidatos</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -1369,11 +1033,6 @@
       <c r="C52">
         <v>11</v>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Disposições Finais</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -1387,12 +1046,6 @@
       <c r="C53">
         <v>5</v>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Disposições
-Transitórias</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -1406,12 +1059,6 @@
       <c r="C54">
         <v>1</v>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Do Direito de
-Resposta</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -1425,12 +1072,6 @@
       <c r="C55">
         <v>10</v>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Do Registro de
-Candidatos</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -1444,15 +1085,6 @@
       <c r="C56">
         <v>2</v>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Do Sistema
-Eletrônico de
-Votação e da
-Totalização dos
-Votos</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -1466,12 +1098,6 @@
       <c r="C57">
         <v>1</v>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Propaganda na
-Internet</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -1485,14 +1111,6 @@
       <c r="C58">
         <v>33</v>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Da Arrecadação
-e da Aplicação
-de Recursos nas
-Campanhas Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -1506,12 +1124,6 @@
       <c r="C59">
         <v>1</v>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Da Prestação de
-Contas</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -1525,12 +1137,6 @@
       <c r="C60">
         <v>7</v>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral em Geral</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -1544,13 +1150,6 @@
       <c r="C61">
         <v>5</v>
       </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Da Propaganda
-Eleitoral no Rádio e
-na Televisão</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -1564,13 +1163,6 @@
       <c r="C62">
         <v>1</v>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Das Convenções
-para a Escolha de
-Candidatos</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -1584,11 +1176,6 @@
       <c r="C63">
         <v>2</v>
       </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Disposições Finais</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -1602,11 +1189,6 @@
       <c r="C64">
         <v>1</v>
       </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Disposições Gerais</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -1620,12 +1202,6 @@
       <c r="C65">
         <v>1</v>
       </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Do Direito de
-Resposta</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -1639,13 +1215,6 @@
       <c r="C66">
         <v>36</v>
       </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Do Fundo Especial
-de Financiamento de
-Campanha (FEFC)</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -1659,12 +1228,6 @@
       <c r="C67">
         <v>3</v>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Do Registro de
-Candidatos</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -1678,12 +1241,6 @@
       <c r="C68">
         <v>14</v>
       </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Propaganda na
-Internet</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -1697,14 +1254,6 @@
       <c r="C69">
         <v>10</v>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Da Arrecadação
-e da Aplicação
-de Recursos nas
-Campanhas Eleitorais</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70">
@@ -1718,12 +1267,6 @@
       <c r="C70">
         <v>1</v>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Da Prestação de
-Contas</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71">
@@ -1737,13 +1280,6 @@
       <c r="C71">
         <v>4</v>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Do Fundo Especial
-de Financiamento de
-Campanha (FEFC)</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72">
@@ -1756,12 +1292,6 @@
       </c>
       <c r="C72">
         <v>4</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Do Registro de
-Candidatos</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>